<commit_message>
Canva- spring:no corresponde a ningun cambio en codigo solo cambio en presentacion
</commit_message>
<xml_diff>
--- a/CRONOGRAMA/Springs.xlsx
+++ b/CRONOGRAMA/Springs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\TALLER DE PROYECTOS\PROYECTO-REPOSITORIO\taller-proyectos-1\CRONOGRAMA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE89A467-9F8C-44AA-BA3A-B4C4F41E9BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AABABB19-116D-44B8-94AF-B45659AD00A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1925,10 +1925,10 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>'Spring 4'!$A$2:$A$5</c:f>
+              <c:f>'Spring 4'!$A$2:$A$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -1946,10 +1946,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Spring 4'!$B$2:$B$5</c:f>
+              <c:f>'Spring 4'!$B$2:$B$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>3</c:v>
                 </c:pt>
@@ -2053,10 +2053,10 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>'Spring 4'!$A$2:$A$5</c:f>
+              <c:f>'Spring 4'!$A$2:$A$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>0</c:v>
                 </c:pt>
@@ -2074,10 +2074,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Spring 4'!$C$2:$C$5</c:f>
+              <c:f>'Spring 4'!$C$2:$C$6</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
                   <c:v>3</c:v>
                 </c:pt>
@@ -2086,6 +2086,9 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2528,8 +2531,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Tabla1345" displayName="Tabla1345" ref="A1:C5" totalsRowShown="0">
-  <autoFilter ref="A1:C5" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Tabla1345" displayName="Tabla1345" ref="A1:C6" totalsRowShown="0">
+  <autoFilter ref="A1:C6" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Tiempo"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Actividad"/>
@@ -3056,6 +3059,9 @@
       <c r="B5" s="4">
         <v>0</v>
       </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>